<commit_message>
Update costing output for 2026-07-31
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CI12"/>
+  <dimension ref="A1:CK12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -643,6 +643,8 @@
     <col width="14" customWidth="1" min="85" max="85"/>
     <col width="14" customWidth="1" min="86" max="86"/>
     <col width="14" customWidth="1" min="87" max="87"/>
+    <col width="14" customWidth="1" min="88" max="88"/>
+    <col width="14" customWidth="1" min="89" max="89"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -909,6 +911,12 @@
         </is>
       </c>
       <c r="CI1" s="3" t="n"/>
+      <c r="CJ1" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CK1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1342,6 +1350,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CJ2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CK2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1693,6 +1711,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CJ3" s="7" t="n">
+        <v>25200</v>
+      </c>
+      <c r="CK3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2044,6 +2070,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CJ4" s="9" t="n">
+        <v>38800</v>
+      </c>
+      <c r="CK4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2309,6 +2343,12 @@
       <c r="CI5" s="7" t="n">
         <v>33300</v>
       </c>
+      <c r="CJ5" s="7" t="n">
+        <v>34200</v>
+      </c>
+      <c r="CK5" s="7" t="n">
+        <v>34400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2660,6 +2700,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CJ6" s="9" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="CK6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3011,6 +3059,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CJ7" s="7" t="n">
+        <v>29400</v>
+      </c>
+      <c r="CK7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3448,6 +3504,16 @@
           <t>2026-07-14</t>
         </is>
       </c>
+      <c r="CJ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="CK8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3713,6 +3779,12 @@
       <c r="CI9" s="13" t="n">
         <v>41300</v>
       </c>
+      <c r="CJ9" s="13" t="n">
+        <v>38400</v>
+      </c>
+      <c r="CK9" s="13" t="n">
+        <v>41600</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3978,6 +4050,12 @@
       <c r="CI10" s="16" t="n">
         <v>-145.94</v>
       </c>
+      <c r="CJ10" s="16" t="n">
+        <v>-1680.09</v>
+      </c>
+      <c r="CK10" s="16" t="n">
+        <v>-1597.66</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4243,6 +4321,12 @@
       <c r="CI11" s="13" t="n">
         <v>43600</v>
       </c>
+      <c r="CJ11" s="13" t="n">
+        <v>40000</v>
+      </c>
+      <c r="CK11" s="13" t="n">
+        <v>44400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4507,6 +4591,12 @@
       </c>
       <c r="CI12" s="16" t="n">
         <v>-557.51</v>
+      </c>
+      <c r="CJ12" s="16" t="n">
+        <v>-2780.73</v>
+      </c>
+      <c r="CK12" s="16" t="n">
+        <v>-1523.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-08-31
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CM12"/>
+  <dimension ref="A1:CO12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -647,6 +647,8 @@
     <col width="14" customWidth="1" min="89" max="89"/>
     <col width="14" customWidth="1" min="90" max="90"/>
     <col width="14" customWidth="1" min="91" max="91"/>
+    <col width="14" customWidth="1" min="92" max="92"/>
+    <col width="14" customWidth="1" min="93" max="93"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -925,6 +927,12 @@
         </is>
       </c>
       <c r="CM1" s="3" t="n"/>
+      <c r="CN1" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="CO1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1378,6 +1386,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CN2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CO2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1745,6 +1763,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CN3" s="7" t="n">
+        <v>29700</v>
+      </c>
+      <c r="CO3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2112,6 +2138,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CN4" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="CO4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2389,6 +2423,12 @@
       <c r="CM5" s="7" t="n">
         <v>35100</v>
       </c>
+      <c r="CN5" s="7" t="n">
+        <v>36500</v>
+      </c>
+      <c r="CO5" s="7" t="n">
+        <v>38900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2756,6 +2796,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CN6" s="9" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="CO6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3123,6 +3171,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CN7" s="7" t="n">
+        <v>33700</v>
+      </c>
+      <c r="CO7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3580,6 +3636,16 @@
           <t>2026-08-18</t>
         </is>
       </c>
+      <c r="CN8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="CO8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3857,6 +3923,12 @@
       <c r="CM9" s="13" t="n">
         <v>42000</v>
       </c>
+      <c r="CN9" s="13" t="n">
+        <v>42500</v>
+      </c>
+      <c r="CO9" s="13" t="n">
+        <v>45800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4134,6 +4206,12 @@
       <c r="CM10" s="16" t="n">
         <v>-2070.98</v>
       </c>
+      <c r="CN10" s="16" t="n">
+        <v>-2309.77</v>
+      </c>
+      <c r="CO10" s="16" t="n">
+        <v>-2059.16</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4411,6 +4489,12 @@
       <c r="CM11" s="13" t="n">
         <v>45100</v>
       </c>
+      <c r="CN11" s="13" t="n">
+        <v>45700</v>
+      </c>
+      <c r="CO11" s="13" t="n">
+        <v>48800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4687,6 +4771,12 @@
       </c>
       <c r="CM12" s="16" t="n">
         <v>-1703.54</v>
+      </c>
+      <c r="CN12" s="16" t="n">
+        <v>-1848.25</v>
+      </c>
+      <c r="CO12" s="16" t="n">
+        <v>-1822.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-08-18
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CK12"/>
+  <dimension ref="A1:CM12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -645,6 +645,8 @@
     <col width="14" customWidth="1" min="87" max="87"/>
     <col width="14" customWidth="1" min="88" max="88"/>
     <col width="14" customWidth="1" min="89" max="89"/>
+    <col width="14" customWidth="1" min="90" max="90"/>
+    <col width="14" customWidth="1" min="91" max="91"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -917,6 +919,12 @@
         </is>
       </c>
       <c r="CK1" s="3" t="n"/>
+      <c r="CL1" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="CM1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1360,6 +1368,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CL2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CM2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1719,6 +1737,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CL3" s="7" t="n">
+        <v>26300</v>
+      </c>
+      <c r="CM3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2078,6 +2104,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CL4" s="9" t="n">
+        <v>38750</v>
+      </c>
+      <c r="CM4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2349,6 +2383,12 @@
       <c r="CK5" s="7" t="n">
         <v>34400</v>
       </c>
+      <c r="CL5" s="7" t="n">
+        <v>34200</v>
+      </c>
+      <c r="CM5" s="7" t="n">
+        <v>35100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2708,6 +2748,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CL6" s="9" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="CM6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3067,6 +3115,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CL7" s="7" t="n">
+        <v>30350</v>
+      </c>
+      <c r="CM7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3514,6 +3570,16 @@
           <t>2026-07-31</t>
         </is>
       </c>
+      <c r="CL8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="CM8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3785,6 +3851,12 @@
       <c r="CK9" s="13" t="n">
         <v>41600</v>
       </c>
+      <c r="CL9" s="13" t="n">
+        <v>39000</v>
+      </c>
+      <c r="CM9" s="13" t="n">
+        <v>42000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4056,6 +4128,12 @@
       <c r="CK10" s="16" t="n">
         <v>-1597.66</v>
       </c>
+      <c r="CL10" s="16" t="n">
+        <v>-2107.8</v>
+      </c>
+      <c r="CM10" s="16" t="n">
+        <v>-2070.98</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4327,6 +4405,12 @@
       <c r="CK11" s="13" t="n">
         <v>44400</v>
       </c>
+      <c r="CL11" s="13" t="n">
+        <v>40900</v>
+      </c>
+      <c r="CM11" s="13" t="n">
+        <v>45100</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4597,6 +4681,12 @@
       </c>
       <c r="CK12" s="16" t="n">
         <v>-1523.24</v>
+      </c>
+      <c r="CL12" s="16" t="n">
+        <v>-2916.67</v>
+      </c>
+      <c r="CM12" s="16" t="n">
+        <v>-1703.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-09-15
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CO12"/>
+  <dimension ref="A1:CQ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -649,6 +649,8 @@
     <col width="14" customWidth="1" min="91" max="91"/>
     <col width="14" customWidth="1" min="92" max="92"/>
     <col width="14" customWidth="1" min="93" max="93"/>
+    <col width="14" customWidth="1" min="94" max="94"/>
+    <col width="14" customWidth="1" min="95" max="95"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -933,6 +935,12 @@
         </is>
       </c>
       <c r="CO1" s="3" t="n"/>
+      <c r="CP1" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="CQ1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1396,6 +1404,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CP2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CQ2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1771,6 +1789,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CP3" s="7" t="n">
+        <v>29600</v>
+      </c>
+      <c r="CQ3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2146,6 +2172,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CP4" s="9" t="n">
+        <v>41700</v>
+      </c>
+      <c r="CQ4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2429,6 +2463,12 @@
       <c r="CO5" s="7" t="n">
         <v>38900</v>
       </c>
+      <c r="CP5" s="7" t="n">
+        <v>37000</v>
+      </c>
+      <c r="CQ5" s="7" t="n">
+        <v>39400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2804,6 +2844,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CP6" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="CQ6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3179,6 +3227,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CP7" s="7" t="n">
+        <v>33800</v>
+      </c>
+      <c r="CQ7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3646,6 +3702,16 @@
           <t>2026-08-31</t>
         </is>
       </c>
+      <c r="CP8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="CQ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3929,6 +3995,12 @@
       <c r="CO9" s="13" t="n">
         <v>45800</v>
       </c>
+      <c r="CP9" s="13" t="n">
+        <v>43600</v>
+      </c>
+      <c r="CQ9" s="13" t="n">
+        <v>47400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4212,6 +4284,12 @@
       <c r="CO10" s="16" t="n">
         <v>-2059.16</v>
       </c>
+      <c r="CP10" s="16" t="n">
+        <v>-1439.38</v>
+      </c>
+      <c r="CQ10" s="16" t="n">
+        <v>-922.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4495,6 +4573,12 @@
       <c r="CO11" s="13" t="n">
         <v>48800</v>
       </c>
+      <c r="CP11" s="13" t="n">
+        <v>46500</v>
+      </c>
+      <c r="CQ11" s="13" t="n">
+        <v>50000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4777,6 +4861,12 @@
       </c>
       <c r="CO12" s="16" t="n">
         <v>-1822.03</v>
+      </c>
+      <c r="CP12" s="16" t="n">
+        <v>-1279.7</v>
+      </c>
+      <c r="CQ12" s="16" t="n">
+        <v>-1088.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-09-23
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ12"/>
+  <dimension ref="A1:CS12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -651,6 +651,8 @@
     <col width="14" customWidth="1" min="93" max="93"/>
     <col width="14" customWidth="1" min="94" max="94"/>
     <col width="14" customWidth="1" min="95" max="95"/>
+    <col width="14" customWidth="1" min="96" max="96"/>
+    <col width="14" customWidth="1" min="97" max="97"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -941,6 +943,12 @@
         </is>
       </c>
       <c r="CQ1" s="3" t="n"/>
+      <c r="CR1" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="CS1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1414,6 +1422,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CR2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CS2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1797,6 +1815,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CR3" s="7" t="n">
+        <v>28100</v>
+      </c>
+      <c r="CS3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2180,6 +2206,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CR4" s="9" t="n">
+        <v>41950</v>
+      </c>
+      <c r="CS4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2469,6 +2503,12 @@
       <c r="CQ5" s="7" t="n">
         <v>39400</v>
       </c>
+      <c r="CR5" s="7" t="n">
+        <v>37400</v>
+      </c>
+      <c r="CS5" s="7" t="n">
+        <v>37800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2852,6 +2892,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CR6" s="9" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="CS6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3235,6 +3283,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CR7" s="7" t="n">
+        <v>32350</v>
+      </c>
+      <c r="CS7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3712,6 +3768,16 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="CR8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="CS8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4001,6 +4067,12 @@
       <c r="CQ9" s="13" t="n">
         <v>47400</v>
       </c>
+      <c r="CR9" s="13" t="n">
+        <v>44000</v>
+      </c>
+      <c r="CS9" s="13" t="n">
+        <v>46850</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4290,6 +4362,12 @@
       <c r="CQ10" s="16" t="n">
         <v>-922.1</v>
       </c>
+      <c r="CR10" s="15" t="n">
+        <v>312.26</v>
+      </c>
+      <c r="CS10" s="15" t="n">
+        <v>28.44</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4579,6 +4657,12 @@
       <c r="CQ11" s="13" t="n">
         <v>50000</v>
       </c>
+      <c r="CR11" s="13" t="n">
+        <v>47100</v>
+      </c>
+      <c r="CS11" s="13" t="n">
+        <v>49800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4867,6 +4951,12 @@
       </c>
       <c r="CQ12" s="16" t="n">
         <v>-1088.67</v>
+      </c>
+      <c r="CR12" s="15" t="n">
+        <v>682.76</v>
+      </c>
+      <c r="CS12" s="15" t="n">
+        <v>223.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-09-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CS12"/>
+  <dimension ref="A1:CU12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -653,6 +653,8 @@
     <col width="14" customWidth="1" min="95" max="95"/>
     <col width="14" customWidth="1" min="96" max="96"/>
     <col width="14" customWidth="1" min="97" max="97"/>
+    <col width="14" customWidth="1" min="98" max="98"/>
+    <col width="14" customWidth="1" min="99" max="99"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -949,6 +951,12 @@
         </is>
       </c>
       <c r="CS1" s="3" t="n"/>
+      <c r="CT1" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CU1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1432,6 +1440,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CT2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CU2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1823,6 +1841,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CT3" s="7" t="n">
+        <v>29300</v>
+      </c>
+      <c r="CU3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2214,6 +2240,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CT4" s="9" t="n">
+        <v>42700</v>
+      </c>
+      <c r="CU4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2509,6 +2543,12 @@
       <c r="CS5" s="7" t="n">
         <v>37800</v>
       </c>
+      <c r="CT5" s="7" t="n">
+        <v>38400</v>
+      </c>
+      <c r="CU5" s="7" t="n">
+        <v>39200</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2900,6 +2940,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CT6" s="9" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="CU6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3291,6 +3339,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CT7" s="7" t="n">
+        <v>34100</v>
+      </c>
+      <c r="CU7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3778,6 +3834,16 @@
           <t>2026-09-23</t>
         </is>
       </c>
+      <c r="CT8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="CU8" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4073,6 +4139,12 @@
       <c r="CS9" s="13" t="n">
         <v>46850</v>
       </c>
+      <c r="CT9" s="13" t="n">
+        <v>45250</v>
+      </c>
+      <c r="CU9" s="13" t="n">
+        <v>48000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4368,6 +4440,12 @@
       <c r="CS10" s="15" t="n">
         <v>28.44</v>
       </c>
+      <c r="CT10" s="15" t="n">
+        <v>89.20999999999999</v>
+      </c>
+      <c r="CU10" s="16" t="n">
+        <v>-268.49</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4663,6 +4741,12 @@
       <c r="CS11" s="13" t="n">
         <v>49800</v>
       </c>
+      <c r="CT11" s="13" t="n">
+        <v>48300</v>
+      </c>
+      <c r="CU11" s="13" t="n">
+        <v>52100</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4957,6 +5041,12 @@
       </c>
       <c r="CS12" s="15" t="n">
         <v>223.87</v>
+      </c>
+      <c r="CT12" s="15" t="n">
+        <v>397.93</v>
+      </c>
+      <c r="CU12" s="15" t="n">
+        <v>1065.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-10-07
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CU12"/>
+  <dimension ref="A1:CW12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -655,6 +655,8 @@
     <col width="14" customWidth="1" min="97" max="97"/>
     <col width="14" customWidth="1" min="98" max="98"/>
     <col width="14" customWidth="1" min="99" max="99"/>
+    <col width="14" customWidth="1" min="100" max="100"/>
+    <col width="14" customWidth="1" min="101" max="101"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -957,6 +959,12 @@
         </is>
       </c>
       <c r="CU1" s="3" t="n"/>
+      <c r="CV1" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="CW1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1450,6 +1458,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CV2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CW2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1849,6 +1867,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CV3" s="7" t="n">
+        <v>29350</v>
+      </c>
+      <c r="CW3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2248,6 +2274,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CV4" s="9" t="n">
+        <v>43000</v>
+      </c>
+      <c r="CW4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2549,6 +2583,12 @@
       <c r="CU5" s="7" t="n">
         <v>39200</v>
       </c>
+      <c r="CV5" s="7" t="n">
+        <v>38400</v>
+      </c>
+      <c r="CW5" s="7" t="n">
+        <v>39500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2948,6 +2988,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CV6" s="9" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="CW6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3347,6 +3395,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CV7" s="7" t="n">
+        <v>34000</v>
+      </c>
+      <c r="CW7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3844,6 +3900,16 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="CV8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="CW8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4145,6 +4211,12 @@
       <c r="CU9" s="13" t="n">
         <v>48000</v>
       </c>
+      <c r="CV9" s="13" t="n">
+        <v>45750</v>
+      </c>
+      <c r="CW9" s="13" t="n">
+        <v>48200</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4446,6 +4518,12 @@
       <c r="CU10" s="16" t="n">
         <v>-268.49</v>
       </c>
+      <c r="CV10" s="15" t="n">
+        <v>483.92</v>
+      </c>
+      <c r="CW10" s="16" t="n">
+        <v>-323.48</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4747,6 +4825,12 @@
       <c r="CU11" s="13" t="n">
         <v>52100</v>
       </c>
+      <c r="CV11" s="13" t="n">
+        <v>48900</v>
+      </c>
+      <c r="CW11" s="13" t="n">
+        <v>53200</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -5047,6 +5131,12 @@
       </c>
       <c r="CU12" s="15" t="n">
         <v>1065.37</v>
+      </c>
+      <c r="CV12" s="15" t="n">
+        <v>891.79</v>
+      </c>
+      <c r="CW12" s="15" t="n">
+        <v>1908.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-10-15
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CW12"/>
+  <dimension ref="A1:CY12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -657,6 +657,8 @@
     <col width="14" customWidth="1" min="99" max="99"/>
     <col width="14" customWidth="1" min="100" max="100"/>
     <col width="14" customWidth="1" min="101" max="101"/>
+    <col width="14" customWidth="1" min="102" max="102"/>
+    <col width="14" customWidth="1" min="103" max="103"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -965,6 +967,12 @@
         </is>
       </c>
       <c r="CW1" s="3" t="n"/>
+      <c r="CX1" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="CY1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1468,6 +1476,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CX2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CY2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1875,6 +1893,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CX3" s="7" t="n">
+        <v>28150</v>
+      </c>
+      <c r="CY3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2282,6 +2308,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CX4" s="9" t="n">
+        <v>42950</v>
+      </c>
+      <c r="CY4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2589,6 +2623,12 @@
       <c r="CW5" s="7" t="n">
         <v>39500</v>
       </c>
+      <c r="CX5" s="7" t="n">
+        <v>37500</v>
+      </c>
+      <c r="CY5" s="7" t="n">
+        <v>37400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2996,6 +3036,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CX6" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="CY6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3403,6 +3451,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CX7" s="7" t="n">
+        <v>32650</v>
+      </c>
+      <c r="CY7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3910,6 +3966,16 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="CX8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="CY8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4217,6 +4283,12 @@
       <c r="CW9" s="13" t="n">
         <v>48200</v>
       </c>
+      <c r="CX9" s="13" t="n">
+        <v>44500</v>
+      </c>
+      <c r="CY9" s="13" t="n">
+        <v>46500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4524,6 +4596,12 @@
       <c r="CW10" s="16" t="n">
         <v>-323.48</v>
       </c>
+      <c r="CX10" s="15" t="n">
+        <v>520.37</v>
+      </c>
+      <c r="CY10" s="16" t="n">
+        <v>-340.54</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4831,6 +4909,12 @@
       <c r="CW11" s="13" t="n">
         <v>53200</v>
       </c>
+      <c r="CX11" s="13" t="n">
+        <v>48300</v>
+      </c>
+      <c r="CY11" s="13" t="n">
+        <v>51400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -5137,6 +5221,12 @@
       </c>
       <c r="CW12" s="15" t="n">
         <v>1908.33</v>
+      </c>
+      <c r="CX12" s="15" t="n">
+        <v>1588.53</v>
+      </c>
+      <c r="CY12" s="15" t="n">
+        <v>1804.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-10-19
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CY12"/>
+  <dimension ref="A1:DA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -659,6 +659,8 @@
     <col width="14" customWidth="1" min="101" max="101"/>
     <col width="14" customWidth="1" min="102" max="102"/>
     <col width="14" customWidth="1" min="103" max="103"/>
+    <col width="14" customWidth="1" min="104" max="104"/>
+    <col width="14" customWidth="1" min="105" max="105"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -973,6 +975,12 @@
         </is>
       </c>
       <c r="CY1" s="3" t="n"/>
+      <c r="CZ1" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="DA1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1486,6 +1494,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CZ2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="DA2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1901,6 +1919,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CZ3" s="7" t="n">
+        <v>27500</v>
+      </c>
+      <c r="DA3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2316,6 +2342,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CZ4" s="9" t="n">
+        <v>42500</v>
+      </c>
+      <c r="DA4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2629,6 +2663,12 @@
       <c r="CY5" s="7" t="n">
         <v>37400</v>
       </c>
+      <c r="CZ5" s="7" t="n">
+        <v>36500</v>
+      </c>
+      <c r="DA5" s="7" t="n">
+        <v>36600</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3044,6 +3084,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CZ6" s="9" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="DA6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3459,6 +3507,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CZ7" s="7" t="n">
+        <v>31900</v>
+      </c>
+      <c r="DA7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3976,6 +4032,16 @@
           <t>2026-10-15</t>
         </is>
       </c>
+      <c r="CZ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="DA8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4289,6 +4355,12 @@
       <c r="CY9" s="13" t="n">
         <v>46500</v>
       </c>
+      <c r="CZ9" s="13" t="n">
+        <v>43700</v>
+      </c>
+      <c r="DA9" s="13" t="n">
+        <v>45900</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4602,6 +4674,12 @@
       <c r="CY10" s="16" t="n">
         <v>-340.54</v>
       </c>
+      <c r="CZ10" s="15" t="n">
+        <v>532.17</v>
+      </c>
+      <c r="DA10" s="16" t="n">
+        <v>-145.36</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4915,6 +4993,12 @@
       <c r="CY11" s="13" t="n">
         <v>51400</v>
       </c>
+      <c r="CZ11" s="13" t="n">
+        <v>47900</v>
+      </c>
+      <c r="DA11" s="13" t="n">
+        <v>50800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -5227,6 +5311,12 @@
       </c>
       <c r="CY12" s="15" t="n">
         <v>1804.74</v>
+      </c>
+      <c r="CZ12" s="15" t="n">
+        <v>2006.82</v>
+      </c>
+      <c r="DA12" s="15" t="n">
+        <v>2006.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-10-21
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DA12"/>
+  <dimension ref="A1:DC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,8 @@
     <col width="14" customWidth="1" min="103" max="103"/>
     <col width="14" customWidth="1" min="104" max="104"/>
     <col width="14" customWidth="1" min="105" max="105"/>
+    <col width="14" customWidth="1" min="106" max="106"/>
+    <col width="14" customWidth="1" min="107" max="107"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -981,6 +983,12 @@
         </is>
       </c>
       <c r="DA1" s="3" t="n"/>
+      <c r="DB1" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="DC1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1504,6 +1512,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="DB2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="DC2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1927,6 +1945,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DB3" s="7" t="n">
+        <v>27800</v>
+      </c>
+      <c r="DC3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2350,6 +2376,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DB4" s="9" t="n">
+        <v>42500</v>
+      </c>
+      <c r="DC4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2669,6 +2703,12 @@
       <c r="DA5" s="7" t="n">
         <v>36600</v>
       </c>
+      <c r="DB5" s="7" t="n">
+        <v>36500</v>
+      </c>
+      <c r="DC5" s="7" t="n">
+        <v>37050</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3092,6 +3132,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DB6" s="9" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="DC6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3515,6 +3563,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DB7" s="7" t="n">
+        <v>32100</v>
+      </c>
+      <c r="DC7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -4042,6 +4098,16 @@
           <t>2026-10-19</t>
         </is>
       </c>
+      <c r="DB8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="DC8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4361,6 +4427,12 @@
       <c r="DA9" s="13" t="n">
         <v>45900</v>
       </c>
+      <c r="DB9" s="13" t="n">
+        <v>44300</v>
+      </c>
+      <c r="DC9" s="13" t="n">
+        <v>46500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4680,6 +4752,12 @@
       <c r="DA10" s="16" t="n">
         <v>-145.36</v>
       </c>
+      <c r="DB10" s="15" t="n">
+        <v>861.76</v>
+      </c>
+      <c r="DC10" s="15" t="n">
+        <v>84.36</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4999,6 +5077,12 @@
       <c r="DA11" s="13" t="n">
         <v>50800</v>
       </c>
+      <c r="DB11" s="13" t="n">
+        <v>48200</v>
+      </c>
+      <c r="DC11" s="13" t="n">
+        <v>51000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -5317,6 +5401,12 @@
       </c>
       <c r="DA12" s="15" t="n">
         <v>2006.27</v>
+      </c>
+      <c r="DB12" s="15" t="n">
+        <v>2034.25</v>
+      </c>
+      <c r="DC12" s="15" t="n">
+        <v>1833.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-10-28
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DC12"/>
+  <dimension ref="A1:DE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,8 @@
     <col width="14" customWidth="1" min="105" max="105"/>
     <col width="14" customWidth="1" min="106" max="106"/>
     <col width="14" customWidth="1" min="107" max="107"/>
+    <col width="14" customWidth="1" min="108" max="108"/>
+    <col width="14" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -989,6 +991,12 @@
         </is>
       </c>
       <c r="DC1" s="3" t="n"/>
+      <c r="DD1" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="DE1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1522,6 +1530,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="DD2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="DE2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1953,6 +1971,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DD3" s="7" t="n">
+        <v>27600</v>
+      </c>
+      <c r="DE3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2384,6 +2410,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DD4" s="9" t="n">
+        <v>42200</v>
+      </c>
+      <c r="DE4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2709,6 +2743,12 @@
       <c r="DC5" s="7" t="n">
         <v>37050</v>
       </c>
+      <c r="DD5" s="7" t="n">
+        <v>35900</v>
+      </c>
+      <c r="DE5" s="7" t="n">
+        <v>36300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3140,6 +3180,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DD6" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="DE6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3571,6 +3619,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="DD7" s="7" t="n">
+        <v>32400</v>
+      </c>
+      <c r="DE7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -4108,6 +4164,16 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="DD8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="DE8" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4433,6 +4499,12 @@
       <c r="DC9" s="13" t="n">
         <v>46500</v>
       </c>
+      <c r="DD9" s="13" t="n">
+        <v>43000</v>
+      </c>
+      <c r="DE9" s="13" t="n">
+        <v>45800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -4758,6 +4830,12 @@
       <c r="DC10" s="15" t="n">
         <v>84.36</v>
       </c>
+      <c r="DD10" s="16" t="n">
+        <v>-191.96</v>
+      </c>
+      <c r="DE10" s="16" t="n">
+        <v>-79.31999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -5083,6 +5161,12 @@
       <c r="DC11" s="13" t="n">
         <v>51000</v>
       </c>
+      <c r="DD11" s="13" t="n">
+        <v>47000</v>
+      </c>
+      <c r="DE11" s="13" t="n">
+        <v>50500</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -5407,6 +5491,12 @@
       </c>
       <c r="DC12" s="15" t="n">
         <v>1833.03</v>
+      </c>
+      <c r="DD12" s="15" t="n">
+        <v>1082.5</v>
+      </c>
+      <c r="DE12" s="15" t="n">
+        <v>1873.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>